<commit_message>
feat: Implement new page object classes for OrangeHRM and DemoQA, enhance test suite organization
- Added `MenuNavigation` class for streamlined navigation in OrangeHRM.
- Introduced `AddEmployeePage` class to manage employee addition functionalities.
- Created `CodeGen` utility for generating Playwright scripts.
- Established `E2ETest` and `PimNewFunctionsTestSuite` for comprehensive testing of new features.
- Developed `DemoQARegressionTestSuite` and `ElementsPageRegressionTest` for regression testing in DemoQA.
- Refactored `ReleasesTestSuite` to include specific tags for better test categorization.
- Removed obsolete `docker-compose.yml` for OrangeHRM setup.
</commit_message>
<xml_diff>
--- a/Playwright/QAPlan_OrangeHRM-PIM_.xlsx
+++ b/Playwright/QAPlan_OrangeHRM-PIM_.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Desktop\Repositorys\QA-Automation-Projects\Playwright\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9486CD47-8A3B-4C5B-B9B4-E4D4A20565DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678293D2-1D47-4544-92FA-AE9490DD77F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{FD97303A-53B3-48AB-ABDA-C3D67ED6805C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" tabRatio="877" firstSheet="6" activeTab="6" xr2:uid="{FD97303A-53B3-48AB-ABDA-C3D67ED6805C}"/>
   </bookViews>
   <sheets>
     <sheet name="Version" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="17" r:id="rId14"/>
+    <pivotCache cacheId="0" r:id="rId14"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="193">
   <si>
     <t xml:space="preserve">OrangeHRM Regression </t>
   </si>
@@ -347,13 +347,6 @@
 Verify deleted user is not able to login;
 Verify hs_hr_employee table and check if details are removed;
 Verify ohrm_user table table and check if details are removed;</t>
-  </si>
-  <si>
-    <t>LC 09/02/26] Need to test with below conditions:
-- 1 Deprecated Fields
-- 1 Country Specific Information
-- 1 Deprecated Fields &amp; 1 Country Specific Information
-- All fields (Deprecated &amp; Country Specific Information)</t>
   </si>
   <si>
     <t>LC 09/02/26] Need to test with below conditions:
@@ -477,9 +470,6 @@
     </r>
   </si>
   <si>
-    <t>LC 09/02/26] Bussiness is not aware how the system should behave then we will proceed with test execution for this TC sharing the results to Bussiness and Dev team</t>
-  </si>
-  <si>
     <t>Verify user should be able to access the system with a Admin account and see Admin and PIM menu options;
 Go to PIM &gt; Reports and click on +Add button; 
 Fill the Report Name Input, add a selection criteria and Display Fields and click on Save;
@@ -746,6 +736,44 @@
   <si>
     <t>Priority Test Cases</t>
   </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>LC 09/02/26] Bussiness is not aware how the system should behave then we will proceed with test execution for this TC sharing the results to Bussiness and Dev team
+LC 17/02/26] Confirmed with Dev and Bussiness and details shouldn't be deleted as the only thing that should be affected is the inputs presented on front end. Marking this Test case as N/A since we already validate in previous test cases;</t>
+  </si>
+  <si>
+    <t>LC 09/02/26] Need to test with below conditions:
+- 1 Deprecated Fields
+- 1 Country Specific Information
+- 1 Deprecated Fields &amp; 1 Country Specific Information
+- All fields (Deprecated &amp; Country Specific Information): Marked as N/A since is redundant</t>
+  </si>
+  <si>
+    <t>TC25_Verify if Admin user upload a csv file with invalid Marital Status value on new employee register then system present a error message</t>
+  </si>
+  <si>
+    <t>TC24_Verify if Admin user upload a csv file with invalid Nationality value on new employee register then system present a error message</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Import is failing and the error message is not friendly user</t>
+  </si>
+  <si>
+    <t>TC18_Verify if Admin user upload a csv file with invalid Nationality value on new employee register then system present a error message</t>
+  </si>
+  <si>
+    <t>TC19_Verify if Admin user upload a csv file with invalid Matrial Status value on new employee register then system present a error message</t>
+  </si>
 </sst>
 </file>
 
@@ -753,7 +781,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
-    <numFmt numFmtId="175" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -1705,69 +1733,6 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="42" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="46" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="47" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="43" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="44" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1940,125 +1905,101 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="46" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="47" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="43" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="44" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Cor1" xfId="1" builtinId="29"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="19">
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <alignment vertical="center"/>
@@ -2288,49 +2229,7 @@
           <a:sp3d/>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent1">
-                    <a:satMod val="103000"/>
-                    <a:lumMod val="102000"/>
-                    <a:tint val="94000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent1">
-                    <a:satMod val="110000"/>
-                    <a:lumMod val="100000"/>
-                    <a:shade val="100000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="99000"/>
-                    <a:satMod val="120000"/>
-                    <a:shade val="78000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -2415,49 +2314,7 @@
           <a:sp3d/>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent2">
-                    <a:satMod val="103000"/>
-                    <a:lumMod val="102000"/>
-                    <a:tint val="94000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent2">
-                    <a:satMod val="110000"/>
-                    <a:lumMod val="100000"/>
-                    <a:shade val="100000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent2">
-                    <a:lumMod val="99000"/>
-                    <a:satMod val="120000"/>
-                    <a:shade val="78000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -2542,49 +2399,7 @@
           <a:sp3d/>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent3">
-                    <a:satMod val="103000"/>
-                    <a:lumMod val="102000"/>
-                    <a:tint val="94000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent3">
-                    <a:satMod val="110000"/>
-                    <a:lumMod val="100000"/>
-                    <a:shade val="100000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent3">
-                    <a:lumMod val="99000"/>
-                    <a:satMod val="120000"/>
-                    <a:shade val="78000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -3706,7 +3521,8 @@
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </chartsheet>
 </file>
 
@@ -3714,7 +3530,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="9294725" cy="6070879"/>
+    <xdr:ext cx="9298075" cy="6072554"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Gráfico 1">
@@ -3746,7 +3562,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="lucas bez" refreshedDate="46078.577163425929" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="23" xr:uid="{CF9BF033-437E-4226-958A-6B15D67E67EC}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:E24" sheet="Low Test Design V1.0"/>
+    <worksheetSource ref="A1:D24" sheet="Low Test Design V1.0"/>
   </cacheSource>
   <cacheFields count="5">
     <cacheField name="App" numFmtId="0">
@@ -3980,7 +3796,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F5C3CF8F-A20B-453B-B450-B603B813E7DC}" name="Tabela Dinâmica4" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F5C3CF8F-A20B-453B-B450-B603B813E7DC}" name="Tabela Dinâmica4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
   <location ref="F1:J8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField showAll="0"/>
@@ -4076,64 +3892,64 @@
     <dataField name="Contagem de Test Scenario" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="16">
-    <format dxfId="28">
+    <format dxfId="18">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format dxfId="17">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="16">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="15">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="27">
+    <format dxfId="14">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="26">
+    <format dxfId="13">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="12">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="11">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="10">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="9">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="21">
+    <format dxfId="8">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="20">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="6">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="5">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="4">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="3">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -4549,28 +4365,28 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="106" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="42"/>
+      <c r="C2" s="107"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="108"/>
     </row>
     <row r="3" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="43"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="45"/>
+      <c r="B3" s="109"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="111"/>
     </row>
     <row r="4" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="C4" s="46">
+      <c r="C4" s="112">
         <v>46022</v>
       </c>
-      <c r="D4" s="47"/>
-      <c r="E4" s="48"/>
+      <c r="D4" s="113"/>
+      <c r="E4" s="114"/>
     </row>
     <row r="5" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="28" t="s">
@@ -4631,88 +4447,88 @@
       <c r="E11" s="38"/>
     </row>
     <row r="12" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="49" t="s">
+      <c r="B12" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="50"/>
-      <c r="D12" s="50"/>
-      <c r="E12" s="51"/>
+      <c r="C12" s="116"/>
+      <c r="D12" s="116"/>
+      <c r="E12" s="117"/>
     </row>
     <row r="13" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="52" t="s">
+      <c r="C13" s="118" t="s">
         <v>4</v>
       </c>
-      <c r="D13" s="52"/>
-      <c r="E13" s="53"/>
+      <c r="D13" s="118"/>
+      <c r="E13" s="119"/>
     </row>
     <row r="14" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="22">
         <v>1</v>
       </c>
-      <c r="C14" s="54" t="s">
+      <c r="C14" s="120" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="55"/>
-      <c r="E14" s="56"/>
+      <c r="D14" s="121"/>
+      <c r="E14" s="122"/>
     </row>
     <row r="15" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="22">
         <v>2</v>
       </c>
-      <c r="C15" s="57"/>
-      <c r="D15" s="57"/>
-      <c r="E15" s="58"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
     </row>
     <row r="16" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="22">
         <v>3</v>
       </c>
-      <c r="C16" s="57"/>
-      <c r="D16" s="57"/>
-      <c r="E16" s="58"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
     </row>
     <row r="17" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="22">
         <v>4</v>
       </c>
-      <c r="C17" s="57"/>
-      <c r="D17" s="57"/>
-      <c r="E17" s="58"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
     </row>
     <row r="18" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="22">
         <v>5</v>
       </c>
-      <c r="C18" s="57"/>
-      <c r="D18" s="57"/>
-      <c r="E18" s="58"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
     </row>
     <row r="19" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="23">
         <v>6</v>
       </c>
-      <c r="C19" s="59"/>
-      <c r="D19" s="59"/>
-      <c r="E19" s="60"/>
+      <c r="C19" s="104"/>
+      <c r="D19" s="104"/>
+      <c r="E19" s="105"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B2:E3"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C14:E14"/>
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="C18:E18"/>
     <mergeCell ref="C19:E19"/>
-    <mergeCell ref="B2:E3"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C14:E14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4735,29 +4551,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="16" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="67" t="s">
+      <c r="B1" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="68" t="s">
+      <c r="C1" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="68" t="s">
+      <c r="D1" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="66" t="s">
+      <c r="E1" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="67" t="s">
+      <c r="F1" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="69" t="s">
+      <c r="G1" s="48" t="s">
         <v>62</v>
       </c>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
@@ -4852,7 +4668,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -4902,64 +4718,64 @@
     <col min="1" max="1" width="17.5703125" style="12" customWidth="1"/>
     <col min="2" max="2" width="13.140625" style="21" customWidth="1"/>
     <col min="3" max="3" width="15.5703125" style="21" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" style="109" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="112"/>
-    <col min="6" max="6" width="26.140625" style="110" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" style="88" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="91"/>
+    <col min="6" max="6" width="26.140625" style="89" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.42578125" style="12" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="4.5703125" style="12" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.28515625" style="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" style="109" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="112"/>
-    <col min="12" max="13" width="24" style="110" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="88" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" style="91"/>
+    <col min="12" max="13" width="24" style="89" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="96" customFormat="1" ht="48" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="96" t="s">
+    <row r="1" spans="1:13" s="75" customFormat="1" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="75" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="96" t="s">
+      <c r="B1" s="75" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="96" t="s">
+      <c r="C1" s="75" t="s">
         <v>58</v>
       </c>
-      <c r="D1" s="108" t="s">
+      <c r="D1" s="87" t="s">
         <v>59</v>
       </c>
-      <c r="E1" s="111"/>
-      <c r="F1" s="119" t="s">
-        <v>180</v>
-      </c>
-      <c r="G1" s="120" t="s">
+      <c r="E1" s="90"/>
+      <c r="F1" s="98" t="s">
         <v>178</v>
+      </c>
+      <c r="G1" s="99" t="s">
+        <v>176</v>
       </c>
       <c r="H1"/>
       <c r="I1"/>
       <c r="J1"/>
-      <c r="K1" s="111"/>
-      <c r="L1" s="113" t="s">
-        <v>183</v>
-      </c>
-      <c r="M1" s="113" t="s">
-        <v>182</v>
+      <c r="K1" s="90"/>
+      <c r="L1" s="92" t="s">
+        <v>181</v>
+      </c>
+      <c r="M1" s="92" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="115">
+      <c r="B2" s="94">
         <v>46069</v>
       </c>
-      <c r="C2" s="115">
+      <c r="C2" s="94">
         <v>46087</v>
       </c>
-      <c r="D2" s="117">
+      <c r="D2" s="96">
         <f>NETWORKDAYS(B2,C2)</f>
         <v>15</v>
       </c>
-      <c r="F2" s="119" t="s">
-        <v>181</v>
+      <c r="F2" s="98" t="s">
+        <v>179</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>14</v>
@@ -4971,148 +4787,148 @@
         <v>18</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="L2" s="114" t="s">
+        <v>177</v>
+      </c>
+      <c r="L2" s="93" t="s">
         <v>14</v>
       </c>
-      <c r="M2" s="122">
+      <c r="M2" s="101">
         <f>GETPIVOTDATA("Test Scenario",$F$1,"Priority","High")/$D$2</f>
         <v>0.8666666666666667</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>121</v>
-      </c>
-      <c r="B3" s="116">
+        <v>119</v>
+      </c>
+      <c r="B3" s="95">
         <v>46067</v>
       </c>
-      <c r="C3" s="115">
+      <c r="C3" s="94">
         <v>46087</v>
       </c>
-      <c r="D3" s="117">
+      <c r="D3" s="96">
         <f t="shared" ref="D3:D4" si="0">NETWORKDAYS(B3,C3)</f>
         <v>15</v>
       </c>
-      <c r="F3" s="107" t="s">
-        <v>132</v>
-      </c>
-      <c r="G3" s="118">
+      <c r="F3" s="86" t="s">
+        <v>130</v>
+      </c>
+      <c r="G3" s="97">
         <v>1</v>
       </c>
-      <c r="H3" s="118"/>
-      <c r="I3" s="118">
+      <c r="H3" s="97"/>
+      <c r="I3" s="97">
         <v>6</v>
       </c>
-      <c r="J3" s="118">
+      <c r="J3" s="97">
         <v>7</v>
       </c>
-      <c r="L3" s="110" t="s">
+      <c r="L3" s="89" t="s">
         <v>18</v>
       </c>
-      <c r="M3" s="121">
+      <c r="M3" s="100">
         <f>GETPIVOTDATA("Test Scenario",$F$1,"Priority","Medium")/$D$2</f>
         <v>0.4</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="B4" s="116">
+        <v>120</v>
+      </c>
+      <c r="B4" s="95">
         <v>46069</v>
       </c>
-      <c r="C4" s="115">
+      <c r="C4" s="94">
         <v>46087</v>
       </c>
-      <c r="D4" s="117">
+      <c r="D4" s="96">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="F4" s="107" t="s">
-        <v>133</v>
-      </c>
-      <c r="G4" s="118">
+      <c r="F4" s="86" t="s">
+        <v>131</v>
+      </c>
+      <c r="G4" s="97">
         <v>4</v>
       </c>
-      <c r="H4" s="118"/>
-      <c r="I4" s="118"/>
-      <c r="J4" s="118">
+      <c r="H4" s="97"/>
+      <c r="I4" s="97"/>
+      <c r="J4" s="97">
         <v>4</v>
       </c>
-      <c r="L4" s="110" t="s">
+      <c r="L4" s="89" t="s">
         <v>21</v>
       </c>
-      <c r="M4" s="121">
+      <c r="M4" s="100">
         <f>GETPIVOTDATA("Test Scenario",$F$1,"Priority","Low")/$D$2</f>
         <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="21"/>
-      <c r="F5" s="107" t="s">
-        <v>127</v>
-      </c>
-      <c r="G5" s="118">
+      <c r="F5" s="86" t="s">
+        <v>125</v>
+      </c>
+      <c r="G5" s="97">
         <v>5</v>
       </c>
-      <c r="H5" s="118"/>
-      <c r="I5" s="118"/>
-      <c r="J5" s="118">
+      <c r="H5" s="97"/>
+      <c r="I5" s="97"/>
+      <c r="J5" s="97">
         <v>5</v>
       </c>
-      <c r="L5" s="110" t="s">
+      <c r="L5" s="89" t="s">
         <v>57</v>
       </c>
-      <c r="M5" s="122">
+      <c r="M5" s="101">
         <f>GETPIVOTDATA("Test Scenario",$F$1)/$D$2</f>
         <v>1.5333333333333334</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="21"/>
-      <c r="F6" s="107" t="s">
-        <v>131</v>
-      </c>
-      <c r="G6" s="118"/>
-      <c r="H6" s="118">
+      <c r="F6" s="86" t="s">
+        <v>129</v>
+      </c>
+      <c r="G6" s="97"/>
+      <c r="H6" s="97">
         <v>4</v>
       </c>
-      <c r="I6" s="118"/>
-      <c r="J6" s="118">
+      <c r="I6" s="97"/>
+      <c r="J6" s="97">
         <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="21"/>
-      <c r="F7" s="107" t="s">
-        <v>129</v>
-      </c>
-      <c r="G7" s="118">
+      <c r="F7" s="86" t="s">
+        <v>127</v>
+      </c>
+      <c r="G7" s="97">
         <v>3</v>
       </c>
-      <c r="H7" s="118"/>
-      <c r="I7" s="118"/>
-      <c r="J7" s="118">
+      <c r="H7" s="97"/>
+      <c r="I7" s="97"/>
+      <c r="J7" s="97">
         <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="21"/>
-      <c r="F8" s="107" t="s">
-        <v>179</v>
-      </c>
-      <c r="G8" s="118">
+      <c r="F8" s="86" t="s">
+        <v>177</v>
+      </c>
+      <c r="G8" s="97">
         <v>13</v>
       </c>
-      <c r="H8" s="118">
+      <c r="H8" s="97">
         <v>4</v>
       </c>
-      <c r="I8" s="118">
+      <c r="I8" s="97">
         <v>6</v>
       </c>
-      <c r="J8" s="118">
+      <c r="J8" s="97">
         <v>23</v>
       </c>
     </row>
@@ -5154,6 +4970,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -5171,26 +4988,26 @@
     <col min="4" max="4" width="68.5703125" style="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="97" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="96" t="s">
+    <row r="1" spans="1:4" s="76" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="96" t="s">
+      <c r="B1" s="75" t="s">
         <v>54</v>
       </c>
-      <c r="C1" s="96" t="s">
+      <c r="C1" s="75" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="96" t="s">
+      <c r="D1" s="75" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C2" s="11" t="s">
         <v>47</v>
@@ -5227,714 +5044,714 @@
   <dimension ref="A1:G70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="86" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" style="87" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" style="87" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" style="87" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" style="87" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="77.5703125" style="91" customWidth="1"/>
-    <col min="7" max="7" width="76.7109375" style="95" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" style="65" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="66" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" style="66" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5703125" style="66" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" style="66" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="77.5703125" style="70" customWidth="1"/>
+    <col min="7" max="7" width="76.7109375" style="74" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="97" customFormat="1" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="104" t="s">
+    <row r="1" spans="1:7" s="76" customFormat="1" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="83" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="105" t="s">
+      <c r="B1" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="105" t="s">
+      <c r="C1" s="84" t="s">
+        <v>149</v>
+      </c>
+      <c r="D1" s="84" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="84" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="84" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="85" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="60">
+        <v>46058</v>
+      </c>
+      <c r="B2" s="61" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="61" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" s="61" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="61" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="67" t="s">
+        <v>146</v>
+      </c>
+      <c r="G2" s="71" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="60">
+        <v>46058</v>
+      </c>
+      <c r="B3" s="62" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="63" t="s">
         <v>151</v>
       </c>
-      <c r="D1" s="105" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" s="105" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="105" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="106" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="81">
+      <c r="D3" s="62" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="63" t="s">
+        <v>65</v>
+      </c>
+      <c r="F3" s="68" t="s">
+        <v>148</v>
+      </c>
+      <c r="G3" s="72" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="60">
         <v>46058</v>
       </c>
-      <c r="B2" s="82" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="82" t="s">
-        <v>152</v>
-      </c>
-      <c r="D2" s="82" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="82" t="s">
+      <c r="B4" s="62" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="62" t="s">
+        <v>150</v>
+      </c>
+      <c r="D4" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="63" t="s">
         <v>65</v>
       </c>
-      <c r="F2" s="88" t="s">
-        <v>148</v>
-      </c>
-      <c r="G2" s="92" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="81">
+      <c r="F4" s="68" t="s">
+        <v>153</v>
+      </c>
+      <c r="G4" s="72" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="60">
         <v>46058</v>
       </c>
-      <c r="B3" s="83" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="84" t="s">
-        <v>153</v>
-      </c>
-      <c r="D3" s="83" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="84" t="s">
+      <c r="B5" s="62" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="62" t="s">
+        <v>150</v>
+      </c>
+      <c r="D5" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="63" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="89" t="s">
-        <v>150</v>
-      </c>
-      <c r="G3" s="93" t="s">
+      <c r="F5" s="68" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="81">
-        <v>46058</v>
-      </c>
-      <c r="B4" s="83" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="83" t="s">
-        <v>152</v>
-      </c>
-      <c r="D4" s="83" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="84" t="s">
-        <v>65</v>
-      </c>
-      <c r="F4" s="89" t="s">
+      <c r="G5" s="72" t="s">
         <v>155</v>
       </c>
-      <c r="G4" s="93" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="81">
-        <v>46058</v>
-      </c>
-      <c r="B5" s="83" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="83" t="s">
-        <v>152</v>
-      </c>
-      <c r="D5" s="83" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="84" t="s">
-        <v>65</v>
-      </c>
-      <c r="F5" s="89" t="s">
-        <v>156</v>
-      </c>
-      <c r="G5" s="93" t="s">
-        <v>157</v>
-      </c>
     </row>
     <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="85"/>
-      <c r="B6" s="83"/>
-      <c r="C6" s="83"/>
-      <c r="D6" s="83"/>
-      <c r="E6" s="83"/>
-      <c r="F6" s="90"/>
-      <c r="G6" s="94"/>
+      <c r="A6" s="64"/>
+      <c r="B6" s="62"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="73"/>
     </row>
     <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="85"/>
-      <c r="B7" s="83"/>
-      <c r="C7" s="83"/>
-      <c r="D7" s="83"/>
-      <c r="E7" s="83"/>
-      <c r="F7" s="90"/>
-      <c r="G7" s="94"/>
+      <c r="A7" s="64"/>
+      <c r="B7" s="62"/>
+      <c r="C7" s="62"/>
+      <c r="D7" s="62"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="69"/>
+      <c r="G7" s="73"/>
     </row>
     <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="85"/>
-      <c r="B8" s="83"/>
-      <c r="C8" s="83"/>
-      <c r="D8" s="83"/>
-      <c r="E8" s="83"/>
-      <c r="F8" s="90"/>
-      <c r="G8" s="94"/>
+      <c r="A8" s="64"/>
+      <c r="B8" s="62"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="69"/>
+      <c r="G8" s="73"/>
     </row>
     <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="85"/>
-      <c r="B9" s="83"/>
-      <c r="C9" s="83"/>
-      <c r="D9" s="83"/>
-      <c r="E9" s="83"/>
-      <c r="F9" s="90"/>
-      <c r="G9" s="94"/>
+      <c r="A9" s="64"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="62"/>
+      <c r="E9" s="62"/>
+      <c r="F9" s="69"/>
+      <c r="G9" s="73"/>
     </row>
     <row r="10" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="85"/>
-      <c r="B10" s="83"/>
-      <c r="C10" s="83"/>
-      <c r="D10" s="83"/>
-      <c r="E10" s="83"/>
-      <c r="F10" s="90"/>
-      <c r="G10" s="94"/>
+      <c r="A10" s="64"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="73"/>
     </row>
     <row r="11" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="85"/>
-      <c r="B11" s="83"/>
-      <c r="C11" s="83"/>
-      <c r="D11" s="83"/>
-      <c r="E11" s="83"/>
-      <c r="F11" s="90"/>
-      <c r="G11" s="94"/>
+      <c r="A11" s="64"/>
+      <c r="B11" s="62"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="62"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="73"/>
     </row>
     <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="85"/>
-      <c r="B12" s="83"/>
-      <c r="C12" s="83"/>
-      <c r="D12" s="83"/>
-      <c r="E12" s="83"/>
-      <c r="F12" s="90"/>
-      <c r="G12" s="94"/>
+      <c r="A12" s="64"/>
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="69"/>
+      <c r="G12" s="73"/>
     </row>
     <row r="13" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="85"/>
-      <c r="B13" s="83"/>
-      <c r="C13" s="83"/>
-      <c r="D13" s="83"/>
-      <c r="E13" s="83"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="94"/>
+      <c r="A13" s="64"/>
+      <c r="B13" s="62"/>
+      <c r="C13" s="62"/>
+      <c r="D13" s="62"/>
+      <c r="E13" s="62"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="73"/>
     </row>
     <row r="14" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="85"/>
-      <c r="B14" s="83"/>
-      <c r="C14" s="83"/>
-      <c r="D14" s="83"/>
-      <c r="E14" s="83"/>
-      <c r="F14" s="90"/>
-      <c r="G14" s="94"/>
+      <c r="A14" s="64"/>
+      <c r="B14" s="62"/>
+      <c r="C14" s="62"/>
+      <c r="D14" s="62"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="69"/>
+      <c r="G14" s="73"/>
     </row>
     <row r="15" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="85"/>
-      <c r="B15" s="83"/>
-      <c r="C15" s="83"/>
-      <c r="D15" s="83"/>
-      <c r="E15" s="83"/>
-      <c r="F15" s="90"/>
-      <c r="G15" s="94"/>
+      <c r="A15" s="64"/>
+      <c r="B15" s="62"/>
+      <c r="C15" s="62"/>
+      <c r="D15" s="62"/>
+      <c r="E15" s="62"/>
+      <c r="F15" s="69"/>
+      <c r="G15" s="73"/>
     </row>
     <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="85"/>
-      <c r="B16" s="83"/>
-      <c r="C16" s="83"/>
-      <c r="D16" s="83"/>
-      <c r="E16" s="83"/>
-      <c r="F16" s="90"/>
-      <c r="G16" s="94"/>
+      <c r="A16" s="64"/>
+      <c r="B16" s="62"/>
+      <c r="C16" s="62"/>
+      <c r="D16" s="62"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="69"/>
+      <c r="G16" s="73"/>
     </row>
     <row r="17" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="85"/>
-      <c r="B17" s="83"/>
-      <c r="C17" s="83"/>
-      <c r="D17" s="83"/>
-      <c r="E17" s="83"/>
-      <c r="F17" s="90"/>
-      <c r="G17" s="94"/>
+      <c r="A17" s="64"/>
+      <c r="B17" s="62"/>
+      <c r="C17" s="62"/>
+      <c r="D17" s="62"/>
+      <c r="E17" s="62"/>
+      <c r="F17" s="69"/>
+      <c r="G17" s="73"/>
     </row>
     <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="85"/>
-      <c r="B18" s="83"/>
-      <c r="C18" s="83"/>
-      <c r="D18" s="83"/>
-      <c r="E18" s="83"/>
-      <c r="F18" s="90"/>
-      <c r="G18" s="94"/>
+      <c r="A18" s="64"/>
+      <c r="B18" s="62"/>
+      <c r="C18" s="62"/>
+      <c r="D18" s="62"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="69"/>
+      <c r="G18" s="73"/>
     </row>
     <row r="19" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="85"/>
-      <c r="B19" s="83"/>
-      <c r="C19" s="83"/>
-      <c r="D19" s="83"/>
-      <c r="E19" s="83"/>
-      <c r="F19" s="90"/>
-      <c r="G19" s="94"/>
+      <c r="A19" s="64"/>
+      <c r="B19" s="62"/>
+      <c r="C19" s="62"/>
+      <c r="D19" s="62"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="69"/>
+      <c r="G19" s="73"/>
     </row>
     <row r="20" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="85"/>
-      <c r="B20" s="83"/>
-      <c r="C20" s="83"/>
-      <c r="D20" s="83"/>
-      <c r="E20" s="83"/>
-      <c r="F20" s="90"/>
-      <c r="G20" s="94"/>
+      <c r="A20" s="64"/>
+      <c r="B20" s="62"/>
+      <c r="C20" s="62"/>
+      <c r="D20" s="62"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="69"/>
+      <c r="G20" s="73"/>
     </row>
     <row r="21" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="85"/>
-      <c r="B21" s="83"/>
-      <c r="C21" s="83"/>
-      <c r="D21" s="83"/>
-      <c r="E21" s="83"/>
-      <c r="F21" s="90"/>
-      <c r="G21" s="94"/>
+      <c r="A21" s="64"/>
+      <c r="B21" s="62"/>
+      <c r="C21" s="62"/>
+      <c r="D21" s="62"/>
+      <c r="E21" s="62"/>
+      <c r="F21" s="69"/>
+      <c r="G21" s="73"/>
     </row>
     <row r="22" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="85"/>
-      <c r="B22" s="83"/>
-      <c r="C22" s="83"/>
-      <c r="D22" s="83"/>
-      <c r="E22" s="83"/>
-      <c r="F22" s="90"/>
-      <c r="G22" s="94"/>
+      <c r="A22" s="64"/>
+      <c r="B22" s="62"/>
+      <c r="C22" s="62"/>
+      <c r="D22" s="62"/>
+      <c r="E22" s="62"/>
+      <c r="F22" s="69"/>
+      <c r="G22" s="73"/>
     </row>
     <row r="23" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="85"/>
-      <c r="B23" s="83"/>
-      <c r="C23" s="83"/>
-      <c r="D23" s="83"/>
-      <c r="E23" s="83"/>
-      <c r="F23" s="90"/>
-      <c r="G23" s="94"/>
+      <c r="A23" s="64"/>
+      <c r="B23" s="62"/>
+      <c r="C23" s="62"/>
+      <c r="D23" s="62"/>
+      <c r="E23" s="62"/>
+      <c r="F23" s="69"/>
+      <c r="G23" s="73"/>
     </row>
     <row r="24" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="85"/>
-      <c r="B24" s="83"/>
-      <c r="C24" s="83"/>
-      <c r="D24" s="83"/>
-      <c r="E24" s="83"/>
-      <c r="F24" s="90"/>
-      <c r="G24" s="94"/>
+      <c r="A24" s="64"/>
+      <c r="B24" s="62"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="62"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="69"/>
+      <c r="G24" s="73"/>
     </row>
     <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="85"/>
-      <c r="B25" s="83"/>
-      <c r="C25" s="83"/>
-      <c r="D25" s="83"/>
-      <c r="E25" s="83"/>
-      <c r="F25" s="90"/>
-      <c r="G25" s="94"/>
+      <c r="A25" s="64"/>
+      <c r="B25" s="62"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="62"/>
+      <c r="F25" s="69"/>
+      <c r="G25" s="73"/>
     </row>
     <row r="26" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="85"/>
-      <c r="B26" s="83"/>
-      <c r="C26" s="83"/>
-      <c r="D26" s="83"/>
-      <c r="E26" s="83"/>
-      <c r="F26" s="90"/>
-      <c r="G26" s="94"/>
+      <c r="A26" s="64"/>
+      <c r="B26" s="62"/>
+      <c r="C26" s="62"/>
+      <c r="D26" s="62"/>
+      <c r="E26" s="62"/>
+      <c r="F26" s="69"/>
+      <c r="G26" s="73"/>
     </row>
     <row r="27" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="85"/>
-      <c r="B27" s="83"/>
-      <c r="C27" s="83"/>
-      <c r="D27" s="83"/>
-      <c r="E27" s="83"/>
-      <c r="F27" s="90"/>
-      <c r="G27" s="94"/>
+      <c r="A27" s="64"/>
+      <c r="B27" s="62"/>
+      <c r="C27" s="62"/>
+      <c r="D27" s="62"/>
+      <c r="E27" s="62"/>
+      <c r="F27" s="69"/>
+      <c r="G27" s="73"/>
     </row>
     <row r="28" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="85"/>
-      <c r="B28" s="83"/>
-      <c r="C28" s="83"/>
-      <c r="D28" s="83"/>
-      <c r="E28" s="83"/>
-      <c r="F28" s="90"/>
-      <c r="G28" s="94"/>
+      <c r="A28" s="64"/>
+      <c r="B28" s="62"/>
+      <c r="C28" s="62"/>
+      <c r="D28" s="62"/>
+      <c r="E28" s="62"/>
+      <c r="F28" s="69"/>
+      <c r="G28" s="73"/>
     </row>
     <row r="29" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="85"/>
-      <c r="B29" s="83"/>
-      <c r="C29" s="83"/>
-      <c r="D29" s="83"/>
-      <c r="E29" s="83"/>
-      <c r="F29" s="90"/>
-      <c r="G29" s="94"/>
+      <c r="A29" s="64"/>
+      <c r="B29" s="62"/>
+      <c r="C29" s="62"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="69"/>
+      <c r="G29" s="73"/>
     </row>
     <row r="30" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="85"/>
-      <c r="B30" s="83"/>
-      <c r="C30" s="83"/>
-      <c r="D30" s="83"/>
-      <c r="E30" s="83"/>
-      <c r="F30" s="90"/>
-      <c r="G30" s="94"/>
+      <c r="A30" s="64"/>
+      <c r="B30" s="62"/>
+      <c r="C30" s="62"/>
+      <c r="D30" s="62"/>
+      <c r="E30" s="62"/>
+      <c r="F30" s="69"/>
+      <c r="G30" s="73"/>
     </row>
     <row r="31" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="85"/>
-      <c r="B31" s="83"/>
-      <c r="C31" s="83"/>
-      <c r="D31" s="83"/>
-      <c r="E31" s="83"/>
-      <c r="F31" s="90"/>
-      <c r="G31" s="94"/>
+      <c r="A31" s="64"/>
+      <c r="B31" s="62"/>
+      <c r="C31" s="62"/>
+      <c r="D31" s="62"/>
+      <c r="E31" s="62"/>
+      <c r="F31" s="69"/>
+      <c r="G31" s="73"/>
     </row>
     <row r="32" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="85"/>
-      <c r="B32" s="83"/>
-      <c r="C32" s="83"/>
-      <c r="D32" s="83"/>
-      <c r="E32" s="83"/>
-      <c r="F32" s="90"/>
-      <c r="G32" s="94"/>
+      <c r="A32" s="64"/>
+      <c r="B32" s="62"/>
+      <c r="C32" s="62"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="69"/>
+      <c r="G32" s="73"/>
     </row>
     <row r="33" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="85"/>
-      <c r="B33" s="83"/>
-      <c r="C33" s="83"/>
-      <c r="D33" s="83"/>
-      <c r="E33" s="83"/>
-      <c r="F33" s="90"/>
-      <c r="G33" s="94"/>
+      <c r="A33" s="64"/>
+      <c r="B33" s="62"/>
+      <c r="C33" s="62"/>
+      <c r="D33" s="62"/>
+      <c r="E33" s="62"/>
+      <c r="F33" s="69"/>
+      <c r="G33" s="73"/>
     </row>
     <row r="34" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="85"/>
-      <c r="B34" s="83"/>
-      <c r="C34" s="83"/>
-      <c r="D34" s="83"/>
-      <c r="E34" s="83"/>
-      <c r="F34" s="90"/>
-      <c r="G34" s="94"/>
+      <c r="A34" s="64"/>
+      <c r="B34" s="62"/>
+      <c r="C34" s="62"/>
+      <c r="D34" s="62"/>
+      <c r="E34" s="62"/>
+      <c r="F34" s="69"/>
+      <c r="G34" s="73"/>
     </row>
     <row r="35" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="85"/>
-      <c r="B35" s="83"/>
-      <c r="C35" s="83"/>
-      <c r="D35" s="83"/>
-      <c r="E35" s="83"/>
-      <c r="F35" s="90"/>
-      <c r="G35" s="94"/>
+      <c r="A35" s="64"/>
+      <c r="B35" s="62"/>
+      <c r="C35" s="62"/>
+      <c r="D35" s="62"/>
+      <c r="E35" s="62"/>
+      <c r="F35" s="69"/>
+      <c r="G35" s="73"/>
     </row>
     <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="85"/>
-      <c r="B36" s="83"/>
-      <c r="C36" s="83"/>
-      <c r="D36" s="83"/>
-      <c r="E36" s="83"/>
-      <c r="F36" s="90"/>
-      <c r="G36" s="94"/>
+      <c r="A36" s="64"/>
+      <c r="B36" s="62"/>
+      <c r="C36" s="62"/>
+      <c r="D36" s="62"/>
+      <c r="E36" s="62"/>
+      <c r="F36" s="69"/>
+      <c r="G36" s="73"/>
     </row>
     <row r="37" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" s="85"/>
-      <c r="B37" s="83"/>
-      <c r="C37" s="83"/>
-      <c r="D37" s="83"/>
-      <c r="E37" s="83"/>
-      <c r="F37" s="90"/>
-      <c r="G37" s="94"/>
+      <c r="A37" s="64"/>
+      <c r="B37" s="62"/>
+      <c r="C37" s="62"/>
+      <c r="D37" s="62"/>
+      <c r="E37" s="62"/>
+      <c r="F37" s="69"/>
+      <c r="G37" s="73"/>
     </row>
     <row r="38" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A38" s="85"/>
-      <c r="B38" s="83"/>
-      <c r="C38" s="83"/>
-      <c r="D38" s="83"/>
-      <c r="E38" s="83"/>
-      <c r="F38" s="90"/>
-      <c r="G38" s="94"/>
+      <c r="A38" s="64"/>
+      <c r="B38" s="62"/>
+      <c r="C38" s="62"/>
+      <c r="D38" s="62"/>
+      <c r="E38" s="62"/>
+      <c r="F38" s="69"/>
+      <c r="G38" s="73"/>
     </row>
     <row r="39" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A39" s="85"/>
-      <c r="B39" s="83"/>
-      <c r="C39" s="83"/>
-      <c r="D39" s="83"/>
-      <c r="E39" s="83"/>
-      <c r="F39" s="90"/>
-      <c r="G39" s="94"/>
+      <c r="A39" s="64"/>
+      <c r="B39" s="62"/>
+      <c r="C39" s="62"/>
+      <c r="D39" s="62"/>
+      <c r="E39" s="62"/>
+      <c r="F39" s="69"/>
+      <c r="G39" s="73"/>
     </row>
     <row r="40" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="85"/>
-      <c r="B40" s="83"/>
-      <c r="C40" s="83"/>
-      <c r="D40" s="83"/>
-      <c r="E40" s="83"/>
-      <c r="F40" s="90"/>
-      <c r="G40" s="94"/>
+      <c r="A40" s="64"/>
+      <c r="B40" s="62"/>
+      <c r="C40" s="62"/>
+      <c r="D40" s="62"/>
+      <c r="E40" s="62"/>
+      <c r="F40" s="69"/>
+      <c r="G40" s="73"/>
     </row>
     <row r="41" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="85"/>
-      <c r="B41" s="83"/>
-      <c r="C41" s="83"/>
-      <c r="D41" s="83"/>
-      <c r="E41" s="83"/>
-      <c r="F41" s="90"/>
-      <c r="G41" s="94"/>
+      <c r="A41" s="64"/>
+      <c r="B41" s="62"/>
+      <c r="C41" s="62"/>
+      <c r="D41" s="62"/>
+      <c r="E41" s="62"/>
+      <c r="F41" s="69"/>
+      <c r="G41" s="73"/>
     </row>
     <row r="42" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="85"/>
-      <c r="B42" s="83"/>
-      <c r="C42" s="83"/>
-      <c r="D42" s="83"/>
-      <c r="E42" s="83"/>
-      <c r="F42" s="90"/>
-      <c r="G42" s="94"/>
+      <c r="A42" s="64"/>
+      <c r="B42" s="62"/>
+      <c r="C42" s="62"/>
+      <c r="D42" s="62"/>
+      <c r="E42" s="62"/>
+      <c r="F42" s="69"/>
+      <c r="G42" s="73"/>
     </row>
     <row r="43" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A43" s="85"/>
-      <c r="B43" s="83"/>
-      <c r="C43" s="83"/>
-      <c r="D43" s="83"/>
-      <c r="E43" s="83"/>
-      <c r="F43" s="90"/>
-      <c r="G43" s="94"/>
+      <c r="A43" s="64"/>
+      <c r="B43" s="62"/>
+      <c r="C43" s="62"/>
+      <c r="D43" s="62"/>
+      <c r="E43" s="62"/>
+      <c r="F43" s="69"/>
+      <c r="G43" s="73"/>
     </row>
     <row r="44" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="85"/>
-      <c r="B44" s="83"/>
-      <c r="C44" s="83"/>
-      <c r="D44" s="83"/>
-      <c r="E44" s="83"/>
-      <c r="F44" s="90"/>
-      <c r="G44" s="94"/>
+      <c r="A44" s="64"/>
+      <c r="B44" s="62"/>
+      <c r="C44" s="62"/>
+      <c r="D44" s="62"/>
+      <c r="E44" s="62"/>
+      <c r="F44" s="69"/>
+      <c r="G44" s="73"/>
     </row>
     <row r="45" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A45" s="85"/>
-      <c r="B45" s="83"/>
-      <c r="C45" s="83"/>
-      <c r="D45" s="83"/>
-      <c r="E45" s="83"/>
-      <c r="F45" s="90"/>
-      <c r="G45" s="94"/>
+      <c r="A45" s="64"/>
+      <c r="B45" s="62"/>
+      <c r="C45" s="62"/>
+      <c r="D45" s="62"/>
+      <c r="E45" s="62"/>
+      <c r="F45" s="69"/>
+      <c r="G45" s="73"/>
     </row>
     <row r="46" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A46" s="85"/>
-      <c r="B46" s="83"/>
-      <c r="C46" s="83"/>
-      <c r="D46" s="83"/>
-      <c r="E46" s="83"/>
-      <c r="F46" s="90"/>
-      <c r="G46" s="94"/>
+      <c r="A46" s="64"/>
+      <c r="B46" s="62"/>
+      <c r="C46" s="62"/>
+      <c r="D46" s="62"/>
+      <c r="E46" s="62"/>
+      <c r="F46" s="69"/>
+      <c r="G46" s="73"/>
     </row>
     <row r="47" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A47" s="85"/>
-      <c r="B47" s="83"/>
-      <c r="C47" s="83"/>
-      <c r="D47" s="83"/>
-      <c r="E47" s="83"/>
-      <c r="F47" s="90"/>
-      <c r="G47" s="94"/>
+      <c r="A47" s="64"/>
+      <c r="B47" s="62"/>
+      <c r="C47" s="62"/>
+      <c r="D47" s="62"/>
+      <c r="E47" s="62"/>
+      <c r="F47" s="69"/>
+      <c r="G47" s="73"/>
     </row>
     <row r="48" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A48" s="85"/>
-      <c r="B48" s="83"/>
-      <c r="C48" s="83"/>
-      <c r="D48" s="83"/>
-      <c r="E48" s="83"/>
-      <c r="F48" s="90"/>
-      <c r="G48" s="94"/>
+      <c r="A48" s="64"/>
+      <c r="B48" s="62"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="69"/>
+      <c r="G48" s="73"/>
     </row>
     <row r="49" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A49" s="85"/>
-      <c r="B49" s="83"/>
-      <c r="C49" s="83"/>
-      <c r="D49" s="83"/>
-      <c r="E49" s="83"/>
-      <c r="F49" s="90"/>
-      <c r="G49" s="94"/>
+      <c r="A49" s="64"/>
+      <c r="B49" s="62"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="69"/>
+      <c r="G49" s="73"/>
     </row>
     <row r="50" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A50" s="85"/>
-      <c r="B50" s="83"/>
-      <c r="C50" s="83"/>
-      <c r="D50" s="83"/>
-      <c r="E50" s="83"/>
-      <c r="F50" s="90"/>
-      <c r="G50" s="94"/>
+      <c r="A50" s="64"/>
+      <c r="B50" s="62"/>
+      <c r="C50" s="62"/>
+      <c r="D50" s="62"/>
+      <c r="E50" s="62"/>
+      <c r="F50" s="69"/>
+      <c r="G50" s="73"/>
     </row>
     <row r="51" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A51" s="85"/>
-      <c r="B51" s="83"/>
-      <c r="C51" s="83"/>
-      <c r="D51" s="83"/>
-      <c r="E51" s="83"/>
-      <c r="F51" s="90"/>
-      <c r="G51" s="94"/>
+      <c r="A51" s="64"/>
+      <c r="B51" s="62"/>
+      <c r="C51" s="62"/>
+      <c r="D51" s="62"/>
+      <c r="E51" s="62"/>
+      <c r="F51" s="69"/>
+      <c r="G51" s="73"/>
     </row>
     <row r="52" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A52" s="85"/>
-      <c r="B52" s="83"/>
-      <c r="C52" s="83"/>
-      <c r="D52" s="83"/>
-      <c r="E52" s="83"/>
-      <c r="F52" s="90"/>
-      <c r="G52" s="94"/>
+      <c r="A52" s="64"/>
+      <c r="B52" s="62"/>
+      <c r="C52" s="62"/>
+      <c r="D52" s="62"/>
+      <c r="E52" s="62"/>
+      <c r="F52" s="69"/>
+      <c r="G52" s="73"/>
     </row>
     <row r="53" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A53" s="85"/>
-      <c r="B53" s="83"/>
-      <c r="C53" s="83"/>
-      <c r="D53" s="83"/>
-      <c r="E53" s="83"/>
-      <c r="F53" s="90"/>
-      <c r="G53" s="94"/>
+      <c r="A53" s="64"/>
+      <c r="B53" s="62"/>
+      <c r="C53" s="62"/>
+      <c r="D53" s="62"/>
+      <c r="E53" s="62"/>
+      <c r="F53" s="69"/>
+      <c r="G53" s="73"/>
     </row>
     <row r="54" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="85"/>
-      <c r="B54" s="83"/>
-      <c r="C54" s="83"/>
-      <c r="D54" s="83"/>
-      <c r="E54" s="83"/>
-      <c r="F54" s="90"/>
-      <c r="G54" s="94"/>
+      <c r="A54" s="64"/>
+      <c r="B54" s="62"/>
+      <c r="C54" s="62"/>
+      <c r="D54" s="62"/>
+      <c r="E54" s="62"/>
+      <c r="F54" s="69"/>
+      <c r="G54" s="73"/>
     </row>
     <row r="55" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A55" s="85"/>
-      <c r="B55" s="83"/>
-      <c r="C55" s="83"/>
-      <c r="D55" s="83"/>
-      <c r="E55" s="83"/>
-      <c r="F55" s="90"/>
-      <c r="G55" s="94"/>
+      <c r="A55" s="64"/>
+      <c r="B55" s="62"/>
+      <c r="C55" s="62"/>
+      <c r="D55" s="62"/>
+      <c r="E55" s="62"/>
+      <c r="F55" s="69"/>
+      <c r="G55" s="73"/>
     </row>
     <row r="56" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A56" s="85"/>
-      <c r="B56" s="83"/>
-      <c r="C56" s="83"/>
-      <c r="D56" s="83"/>
-      <c r="E56" s="83"/>
-      <c r="F56" s="90"/>
-      <c r="G56" s="94"/>
+      <c r="A56" s="64"/>
+      <c r="B56" s="62"/>
+      <c r="C56" s="62"/>
+      <c r="D56" s="62"/>
+      <c r="E56" s="62"/>
+      <c r="F56" s="69"/>
+      <c r="G56" s="73"/>
     </row>
     <row r="57" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A57" s="85"/>
-      <c r="B57" s="83"/>
-      <c r="C57" s="83"/>
-      <c r="D57" s="83"/>
-      <c r="E57" s="83"/>
-      <c r="F57" s="90"/>
-      <c r="G57" s="94"/>
+      <c r="A57" s="64"/>
+      <c r="B57" s="62"/>
+      <c r="C57" s="62"/>
+      <c r="D57" s="62"/>
+      <c r="E57" s="62"/>
+      <c r="F57" s="69"/>
+      <c r="G57" s="73"/>
     </row>
     <row r="58" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A58" s="85"/>
-      <c r="B58" s="83"/>
-      <c r="C58" s="83"/>
-      <c r="D58" s="83"/>
-      <c r="E58" s="83"/>
-      <c r="F58" s="90"/>
-      <c r="G58" s="94"/>
+      <c r="A58" s="64"/>
+      <c r="B58" s="62"/>
+      <c r="C58" s="62"/>
+      <c r="D58" s="62"/>
+      <c r="E58" s="62"/>
+      <c r="F58" s="69"/>
+      <c r="G58" s="73"/>
     </row>
     <row r="59" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A59" s="85"/>
-      <c r="B59" s="83"/>
-      <c r="C59" s="83"/>
-      <c r="D59" s="83"/>
-      <c r="E59" s="83"/>
-      <c r="F59" s="90"/>
-      <c r="G59" s="94"/>
+      <c r="A59" s="64"/>
+      <c r="B59" s="62"/>
+      <c r="C59" s="62"/>
+      <c r="D59" s="62"/>
+      <c r="E59" s="62"/>
+      <c r="F59" s="69"/>
+      <c r="G59" s="73"/>
     </row>
     <row r="60" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A60" s="85"/>
-      <c r="B60" s="83"/>
-      <c r="C60" s="83"/>
-      <c r="D60" s="83"/>
-      <c r="E60" s="83"/>
-      <c r="F60" s="90"/>
-      <c r="G60" s="94"/>
+      <c r="A60" s="64"/>
+      <c r="B60" s="62"/>
+      <c r="C60" s="62"/>
+      <c r="D60" s="62"/>
+      <c r="E60" s="62"/>
+      <c r="F60" s="69"/>
+      <c r="G60" s="73"/>
     </row>
     <row r="61" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A61" s="85"/>
-      <c r="B61" s="83"/>
-      <c r="C61" s="83"/>
-      <c r="D61" s="83"/>
-      <c r="E61" s="83"/>
-      <c r="F61" s="90"/>
-      <c r="G61" s="94"/>
+      <c r="A61" s="64"/>
+      <c r="B61" s="62"/>
+      <c r="C61" s="62"/>
+      <c r="D61" s="62"/>
+      <c r="E61" s="62"/>
+      <c r="F61" s="69"/>
+      <c r="G61" s="73"/>
     </row>
     <row r="62" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A62" s="85"/>
-      <c r="B62" s="83"/>
-      <c r="C62" s="83"/>
-      <c r="D62" s="83"/>
-      <c r="E62" s="83"/>
-      <c r="F62" s="90"/>
-      <c r="G62" s="94"/>
+      <c r="A62" s="64"/>
+      <c r="B62" s="62"/>
+      <c r="C62" s="62"/>
+      <c r="D62" s="62"/>
+      <c r="E62" s="62"/>
+      <c r="F62" s="69"/>
+      <c r="G62" s="73"/>
     </row>
     <row r="63" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A63" s="85"/>
-      <c r="B63" s="83"/>
-      <c r="C63" s="83"/>
-      <c r="D63" s="83"/>
-      <c r="E63" s="83"/>
-      <c r="F63" s="90"/>
-      <c r="G63" s="94"/>
+      <c r="A63" s="64"/>
+      <c r="B63" s="62"/>
+      <c r="C63" s="62"/>
+      <c r="D63" s="62"/>
+      <c r="E63" s="62"/>
+      <c r="F63" s="69"/>
+      <c r="G63" s="73"/>
     </row>
     <row r="64" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A64" s="85"/>
-      <c r="B64" s="83"/>
-      <c r="C64" s="83"/>
-      <c r="D64" s="83"/>
-      <c r="E64" s="83"/>
-      <c r="F64" s="90"/>
-      <c r="G64" s="94"/>
+      <c r="A64" s="64"/>
+      <c r="B64" s="62"/>
+      <c r="C64" s="62"/>
+      <c r="D64" s="62"/>
+      <c r="E64" s="62"/>
+      <c r="F64" s="69"/>
+      <c r="G64" s="73"/>
     </row>
     <row r="65" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A65" s="85"/>
-      <c r="B65" s="83"/>
-      <c r="C65" s="83"/>
-      <c r="D65" s="83"/>
-      <c r="E65" s="83"/>
-      <c r="F65" s="90"/>
-      <c r="G65" s="94"/>
+      <c r="A65" s="64"/>
+      <c r="B65" s="62"/>
+      <c r="C65" s="62"/>
+      <c r="D65" s="62"/>
+      <c r="E65" s="62"/>
+      <c r="F65" s="69"/>
+      <c r="G65" s="73"/>
     </row>
     <row r="66" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A66" s="85"/>
-      <c r="B66" s="83"/>
-      <c r="C66" s="83"/>
-      <c r="D66" s="83"/>
-      <c r="E66" s="83"/>
-      <c r="F66" s="90"/>
-      <c r="G66" s="94"/>
+      <c r="A66" s="64"/>
+      <c r="B66" s="62"/>
+      <c r="C66" s="62"/>
+      <c r="D66" s="62"/>
+      <c r="E66" s="62"/>
+      <c r="F66" s="69"/>
+      <c r="G66" s="73"/>
     </row>
     <row r="67" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A67" s="85"/>
-      <c r="B67" s="83"/>
-      <c r="C67" s="83"/>
-      <c r="D67" s="83"/>
-      <c r="E67" s="83"/>
-      <c r="F67" s="90"/>
-      <c r="G67" s="94"/>
+      <c r="A67" s="64"/>
+      <c r="B67" s="62"/>
+      <c r="C67" s="62"/>
+      <c r="D67" s="62"/>
+      <c r="E67" s="62"/>
+      <c r="F67" s="69"/>
+      <c r="G67" s="73"/>
     </row>
     <row r="68" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A68" s="85"/>
-      <c r="B68" s="83"/>
-      <c r="C68" s="83"/>
-      <c r="D68" s="83"/>
-      <c r="E68" s="83"/>
-      <c r="F68" s="90"/>
-      <c r="G68" s="94"/>
+      <c r="A68" s="64"/>
+      <c r="B68" s="62"/>
+      <c r="C68" s="62"/>
+      <c r="D68" s="62"/>
+      <c r="E68" s="62"/>
+      <c r="F68" s="69"/>
+      <c r="G68" s="73"/>
     </row>
     <row r="69" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A69" s="85"/>
-      <c r="B69" s="83"/>
-      <c r="C69" s="83"/>
-      <c r="D69" s="83"/>
-      <c r="E69" s="83"/>
-      <c r="F69" s="90"/>
-      <c r="G69" s="94"/>
+      <c r="A69" s="64"/>
+      <c r="B69" s="62"/>
+      <c r="C69" s="62"/>
+      <c r="D69" s="62"/>
+      <c r="E69" s="62"/>
+      <c r="F69" s="69"/>
+      <c r="G69" s="73"/>
     </row>
     <row r="70" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A70" s="85"/>
-      <c r="B70" s="83"/>
-      <c r="C70" s="83"/>
-      <c r="D70" s="83"/>
-      <c r="E70" s="83"/>
-      <c r="F70" s="90"/>
-      <c r="G70" s="94"/>
+      <c r="A70" s="64"/>
+      <c r="B70" s="62"/>
+      <c r="C70" s="62"/>
+      <c r="D70" s="62"/>
+      <c r="E70" s="62"/>
+      <c r="F70" s="69"/>
+      <c r="G70" s="73"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -5979,16 +5796,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="103" t="s">
+      <c r="A1" s="82" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="103" t="s">
+      <c r="B1" s="82" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="103" t="s">
+      <c r="C1" s="82" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="103" t="s">
+      <c r="D1" s="82" t="s">
         <v>34</v>
       </c>
     </row>
@@ -5997,13 +5814,13 @@
         <v>30</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6011,13 +5828,13 @@
         <v>31</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6025,13 +5842,13 @@
         <v>32</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6134,690 +5951,753 @@
   <dimension ref="A1:K32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="75" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" style="73" customWidth="1"/>
-    <col min="3" max="3" width="58.5703125" style="77" customWidth="1"/>
-    <col min="4" max="4" width="33.85546875" style="74" customWidth="1"/>
-    <col min="5" max="5" width="49.28515625" style="77" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" style="73" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" style="73" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" style="73" customWidth="1"/>
-    <col min="9" max="9" width="18.7109375" style="73" customWidth="1"/>
-    <col min="10" max="10" width="19.42578125" style="73" customWidth="1"/>
-    <col min="11" max="11" width="77.5703125" style="79" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" style="54" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" style="52" customWidth="1"/>
+    <col min="3" max="3" width="58.5703125" style="56" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" style="53" customWidth="1"/>
+    <col min="5" max="5" width="49.28515625" style="56" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" style="52" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" style="52" customWidth="1"/>
+    <col min="8" max="8" width="19.140625" style="52" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" style="52" customWidth="1"/>
+    <col min="10" max="10" width="19.42578125" style="52" customWidth="1"/>
+    <col min="11" max="11" width="77.5703125" style="58" customWidth="1"/>
     <col min="12" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="102" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="98" t="s">
+    <row r="1" spans="1:11" s="81" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="99" t="s">
+      <c r="B1" s="78" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="100" t="s">
+      <c r="C1" s="79" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="100" t="s">
+      <c r="D1" s="79" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="100" t="s">
+      <c r="E1" s="79" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="99" t="s">
+      <c r="F1" s="78" t="s">
         <v>40</v>
       </c>
-      <c r="G1" s="99" t="s">
+      <c r="G1" s="78" t="s">
         <v>41</v>
       </c>
-      <c r="H1" s="99" t="s">
+      <c r="H1" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="99" t="s">
+      <c r="I1" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="99" t="s">
+      <c r="J1" s="78" t="s">
         <v>42</v>
       </c>
-      <c r="K1" s="101" t="s">
+      <c r="K1" s="80" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="225" x14ac:dyDescent="0.25">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="71" t="s">
+      <c r="B2" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="76" t="s">
+      <c r="C2" s="55" t="s">
         <v>72</v>
       </c>
-      <c r="D2" s="72" t="s">
+      <c r="D2" s="51" t="s">
         <v>74</v>
       </c>
-      <c r="E2" s="76" t="s">
+      <c r="E2" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="71">
+      <c r="F2" s="50">
         <v>1</v>
       </c>
-      <c r="G2" s="71" t="s">
+      <c r="G2" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H2" s="71" t="s">
+      <c r="H2" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="71" t="s">
+      <c r="I2" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="71" t="s">
+      <c r="J2" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K2" s="78" t="s">
+      <c r="K2" s="57" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="195" x14ac:dyDescent="0.25">
-      <c r="A3" s="70" t="s">
+      <c r="A3" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B3" s="71" t="s">
+      <c r="B3" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="76" t="s">
+      <c r="C3" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="D3" s="72" t="s">
+      <c r="D3" s="51" t="s">
         <v>74</v>
       </c>
-      <c r="E3" s="76" t="s">
+      <c r="E3" s="55" t="s">
         <v>82</v>
       </c>
-      <c r="F3" s="71">
+      <c r="F3" s="50">
         <v>1</v>
       </c>
-      <c r="G3" s="71" t="s">
+      <c r="G3" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H3" s="71" t="s">
+      <c r="H3" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="71" t="s">
+      <c r="I3" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="71" t="s">
+      <c r="J3" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K3" s="78" t="s">
+      <c r="K3" s="57" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="120" x14ac:dyDescent="0.25">
-      <c r="A4" s="70" t="s">
+      <c r="A4" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B4" s="71" t="s">
+      <c r="B4" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="76" t="s">
+      <c r="C4" s="55" t="s">
         <v>79</v>
       </c>
-      <c r="D4" s="72" t="s">
+      <c r="D4" s="51" t="s">
         <v>74</v>
       </c>
-      <c r="E4" s="76" t="s">
+      <c r="E4" s="55" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="71">
+      <c r="F4" s="50">
         <v>1</v>
       </c>
-      <c r="G4" s="71" t="s">
+      <c r="G4" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="71" t="s">
+      <c r="H4" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="71" t="s">
+      <c r="I4" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="71" t="s">
+      <c r="J4" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K4" s="78"/>
+      <c r="K4" s="57"/>
     </row>
     <row r="5" spans="1:11" ht="120" x14ac:dyDescent="0.25">
-      <c r="A5" s="70" t="s">
+      <c r="A5" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="71" t="s">
+      <c r="B5" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="76" t="s">
+      <c r="C5" s="55" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="72" t="s">
+      <c r="D5" s="51" t="s">
         <v>85</v>
       </c>
-      <c r="E5" s="76" t="s">
+      <c r="E5" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="71">
+      <c r="F5" s="50">
         <v>1</v>
       </c>
-      <c r="G5" s="71" t="s">
+      <c r="G5" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="71" t="s">
+      <c r="H5" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="71" t="s">
+      <c r="I5" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="71" t="s">
+      <c r="J5" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K5" s="78" t="s">
+      <c r="K5" s="57" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="180" x14ac:dyDescent="0.25">
-      <c r="A6" s="70" t="s">
+      <c r="A6" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="71" t="s">
+      <c r="B6" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="76" t="s">
+      <c r="C6" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="D6" s="72" t="s">
+      <c r="D6" s="51" t="s">
         <v>85</v>
       </c>
-      <c r="E6" s="76" t="s">
+      <c r="E6" s="55" t="s">
         <v>88</v>
       </c>
-      <c r="F6" s="71">
+      <c r="F6" s="50">
         <v>1</v>
       </c>
-      <c r="G6" s="71" t="s">
+      <c r="G6" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="71" t="s">
+      <c r="H6" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="71" t="s">
+      <c r="I6" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="71" t="s">
+      <c r="J6" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K6" s="78" t="s">
+      <c r="K6" s="57" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="180" x14ac:dyDescent="0.25">
-      <c r="A7" s="70" t="s">
+      <c r="A7" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="71" t="s">
+      <c r="B7" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="76" t="s">
-        <v>120</v>
-      </c>
-      <c r="D7" s="72" t="s">
+      <c r="C7" s="55" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="51" t="s">
         <v>85</v>
       </c>
-      <c r="E7" s="76" t="s">
+      <c r="E7" s="55" t="s">
+        <v>109</v>
+      </c>
+      <c r="F7" s="50">
+        <v>4</v>
+      </c>
+      <c r="G7" s="50" t="s">
+        <v>76</v>
+      </c>
+      <c r="H7" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="K7" s="57" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="210" x14ac:dyDescent="0.25">
+      <c r="A8" s="49" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="55" t="s">
+        <v>90</v>
+      </c>
+      <c r="D8" s="51" t="s">
+        <v>85</v>
+      </c>
+      <c r="E8" s="55" t="s">
+        <v>108</v>
+      </c>
+      <c r="F8" s="50">
+        <v>2</v>
+      </c>
+      <c r="G8" s="50" t="s">
+        <v>76</v>
+      </c>
+      <c r="H8" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="K8" s="57" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="180" x14ac:dyDescent="0.25">
+      <c r="A9" s="49" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="D9" s="51" t="s">
         <v>110</v>
       </c>
-      <c r="F7" s="71">
-        <v>4</v>
-      </c>
-      <c r="G7" s="71" t="s">
+      <c r="E9" s="55" t="s">
+        <v>117</v>
+      </c>
+      <c r="F9" s="50">
+        <v>2</v>
+      </c>
+      <c r="G9" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H7" s="71" t="s">
+      <c r="H9" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="K9" s="57" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+      <c r="A10" s="49" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="55" t="s">
+        <v>92</v>
+      </c>
+      <c r="D10" s="51" t="s">
+        <v>110</v>
+      </c>
+      <c r="E10" s="55" t="s">
+        <v>111</v>
+      </c>
+      <c r="F10" s="50">
+        <v>2</v>
+      </c>
+      <c r="G10" s="50" t="s">
+        <v>76</v>
+      </c>
+      <c r="H10" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="K10" s="57" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="180" x14ac:dyDescent="0.25">
+      <c r="A11" s="49" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="55" t="s">
+        <v>93</v>
+      </c>
+      <c r="D11" s="51" t="s">
+        <v>110</v>
+      </c>
+      <c r="E11" s="55" t="s">
+        <v>112</v>
+      </c>
+      <c r="F11" s="50">
+        <v>1</v>
+      </c>
+      <c r="G11" s="50" t="s">
+        <v>94</v>
+      </c>
+      <c r="H11" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="I7" s="71" t="s">
-        <v>21</v>
-      </c>
-      <c r="J7" s="71" t="s">
+      <c r="I11" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="J11" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K7" s="78" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="210" x14ac:dyDescent="0.25">
-      <c r="A8" s="70" t="s">
+      <c r="K11" s="57" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="345" x14ac:dyDescent="0.25">
+      <c r="A12" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B8" s="71" t="s">
+      <c r="B12" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="76" t="s">
-        <v>91</v>
-      </c>
-      <c r="D8" s="72" t="s">
+      <c r="C12" s="55" t="s">
+        <v>95</v>
+      </c>
+      <c r="D12" s="51" t="s">
         <v>85</v>
       </c>
-      <c r="E8" s="76" t="s">
-        <v>109</v>
-      </c>
-      <c r="F8" s="71">
-        <v>2</v>
-      </c>
-      <c r="G8" s="71" t="s">
+      <c r="E12" s="55" t="s">
+        <v>113</v>
+      </c>
+      <c r="F12" s="50">
+        <v>1</v>
+      </c>
+      <c r="G12" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="71" t="s">
+      <c r="H12" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="71" t="s">
-        <v>18</v>
-      </c>
-      <c r="J8" s="71" t="s">
+      <c r="I12" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="J12" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K8" s="78" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="180" x14ac:dyDescent="0.25">
-      <c r="A9" s="70" t="s">
+      <c r="K12" s="57" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="360" x14ac:dyDescent="0.25">
+      <c r="A13" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B9" s="71" t="s">
+      <c r="B13" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="76" t="s">
-        <v>92</v>
-      </c>
-      <c r="D9" s="72" t="s">
-        <v>111</v>
-      </c>
-      <c r="E9" s="76" t="s">
-        <v>119</v>
-      </c>
-      <c r="F9" s="71">
-        <v>2</v>
-      </c>
-      <c r="G9" s="71" t="s">
+      <c r="C13" s="55" t="s">
+        <v>96</v>
+      </c>
+      <c r="D13" s="51" t="s">
+        <v>114</v>
+      </c>
+      <c r="E13" s="55" t="s">
+        <v>116</v>
+      </c>
+      <c r="F13" s="50">
+        <v>1</v>
+      </c>
+      <c r="G13" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="71" t="s">
+      <c r="H13" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="71" t="s">
-        <v>18</v>
-      </c>
-      <c r="J9" s="71" t="s">
+      <c r="I13" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="J13" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K9" s="78" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="165" x14ac:dyDescent="0.25">
-      <c r="A10" s="70" t="s">
+      <c r="K13" s="57" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="315" x14ac:dyDescent="0.25">
+      <c r="A14" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B10" s="71" t="s">
+      <c r="B14" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="76" t="s">
-        <v>93</v>
-      </c>
-      <c r="D10" s="72" t="s">
-        <v>111</v>
-      </c>
-      <c r="E10" s="76" t="s">
-        <v>112</v>
-      </c>
-      <c r="F10" s="71">
-        <v>2</v>
-      </c>
-      <c r="G10" s="71" t="s">
+      <c r="C14" s="55" t="s">
+        <v>97</v>
+      </c>
+      <c r="D14" s="51" t="s">
+        <v>114</v>
+      </c>
+      <c r="E14" s="55" t="s">
+        <v>115</v>
+      </c>
+      <c r="F14" s="50">
+        <v>1</v>
+      </c>
+      <c r="G14" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H10" s="71" t="s">
+      <c r="H14" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="71" t="s">
-        <v>18</v>
-      </c>
-      <c r="J10" s="71" t="s">
+      <c r="I14" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="J14" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K10" s="78" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="180" x14ac:dyDescent="0.25">
-      <c r="A11" s="70" t="s">
+      <c r="K14" s="57" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="210" x14ac:dyDescent="0.25">
+      <c r="A15" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B11" s="71" t="s">
+      <c r="B15" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="76" t="s">
-        <v>94</v>
-      </c>
-      <c r="D11" s="72" t="s">
-        <v>111</v>
-      </c>
-      <c r="E11" s="76" t="s">
-        <v>113</v>
-      </c>
-      <c r="F11" s="71">
+      <c r="C15" s="55" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15" s="55" t="s">
+        <v>121</v>
+      </c>
+      <c r="F15" s="50">
         <v>1</v>
       </c>
-      <c r="G11" s="71" t="s">
-        <v>95</v>
-      </c>
-      <c r="H11" s="71" t="s">
+      <c r="G15" s="50" t="s">
+        <v>76</v>
+      </c>
+      <c r="H15" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="J15" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="K15" s="57"/>
+    </row>
+    <row r="16" spans="1:11" ht="210" x14ac:dyDescent="0.25">
+      <c r="A16" s="49" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="55" t="s">
+        <v>101</v>
+      </c>
+      <c r="D16" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="E16" s="55" t="s">
+        <v>122</v>
+      </c>
+      <c r="F16" s="50">
+        <v>1</v>
+      </c>
+      <c r="G16" s="50" t="s">
+        <v>76</v>
+      </c>
+      <c r="H16" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="I11" s="71" t="s">
+      <c r="I16" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="J11" s="71" t="s">
+      <c r="J16" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K11" s="78" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="345" x14ac:dyDescent="0.25">
-      <c r="A12" s="70" t="s">
+      <c r="K16" s="57" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="210" x14ac:dyDescent="0.25">
+      <c r="A17" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="71" t="s">
+      <c r="B17" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="76" t="s">
-        <v>96</v>
-      </c>
-      <c r="D12" s="72" t="s">
-        <v>85</v>
-      </c>
-      <c r="E12" s="76" t="s">
-        <v>115</v>
-      </c>
-      <c r="F12" s="71">
+      <c r="C17" s="55" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="E17" s="55" t="s">
+        <v>122</v>
+      </c>
+      <c r="F17" s="50">
         <v>1</v>
       </c>
-      <c r="G12" s="71" t="s">
+      <c r="G17" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H12" s="71" t="s">
-        <v>17</v>
-      </c>
-      <c r="I12" s="71" t="s">
+      <c r="H17" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="I17" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="71" t="s">
+      <c r="J17" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K12" s="78" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="360" x14ac:dyDescent="0.25">
-      <c r="A13" s="70" t="s">
+      <c r="K17" s="57" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="210" x14ac:dyDescent="0.25">
+      <c r="A18" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="71" t="s">
+      <c r="B18" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="76" t="s">
-        <v>97</v>
-      </c>
-      <c r="D13" s="72" t="s">
-        <v>116</v>
-      </c>
-      <c r="E13" s="76" t="s">
-        <v>118</v>
-      </c>
-      <c r="F13" s="71">
+      <c r="C18" s="55" t="s">
+        <v>102</v>
+      </c>
+      <c r="D18" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="E18" s="55" t="s">
+        <v>122</v>
+      </c>
+      <c r="F18" s="50">
         <v>1</v>
       </c>
-      <c r="G13" s="71" t="s">
+      <c r="G18" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H13" s="71" t="s">
-        <v>17</v>
-      </c>
-      <c r="I13" s="71" t="s">
+      <c r="H18" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="I18" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="71" t="s">
+      <c r="J18" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K13" s="78" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="315" x14ac:dyDescent="0.25">
-      <c r="A14" s="70" t="s">
+      <c r="K18" s="57" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="210" x14ac:dyDescent="0.25">
+      <c r="A19" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B14" s="71" t="s">
+      <c r="B19" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="76" t="s">
-        <v>98</v>
-      </c>
-      <c r="D14" s="72" t="s">
-        <v>116</v>
-      </c>
-      <c r="E14" s="76" t="s">
-        <v>117</v>
-      </c>
-      <c r="F14" s="71">
+      <c r="C19" s="55" t="s">
+        <v>191</v>
+      </c>
+      <c r="D19" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="E19" s="55" t="s">
+        <v>122</v>
+      </c>
+      <c r="F19" s="50">
         <v>1</v>
       </c>
-      <c r="G14" s="71" t="s">
+      <c r="G19" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H14" s="71" t="s">
-        <v>17</v>
-      </c>
-      <c r="I14" s="71" t="s">
+      <c r="H19" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="I19" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="J14" s="71" t="s">
+      <c r="J19" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K14" s="78" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="210" x14ac:dyDescent="0.25">
-      <c r="A15" s="70" t="s">
+      <c r="K19" s="57" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="210" x14ac:dyDescent="0.25">
+      <c r="A20" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="71" t="s">
+      <c r="B20" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="76" t="s">
-        <v>100</v>
-      </c>
-      <c r="D15" s="72" t="s">
-        <v>107</v>
-      </c>
-      <c r="E15" s="76" t="s">
-        <v>123</v>
-      </c>
-      <c r="F15" s="71">
+      <c r="C20" s="55" t="s">
+        <v>192</v>
+      </c>
+      <c r="D20" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="E20" s="55" t="s">
+        <v>122</v>
+      </c>
+      <c r="F20" s="50">
         <v>1</v>
       </c>
-      <c r="G15" s="71" t="s">
+      <c r="G20" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H15" s="71" t="s">
-        <v>17</v>
-      </c>
-      <c r="I15" s="71" t="s">
+      <c r="H20" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="I20" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="J15" s="71" t="s">
+      <c r="J20" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="K15" s="78"/>
-    </row>
-    <row r="16" spans="1:11" ht="210" x14ac:dyDescent="0.25">
-      <c r="A16" s="70" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="C16" s="76" t="s">
-        <v>102</v>
-      </c>
-      <c r="D16" s="72" t="s">
-        <v>107</v>
-      </c>
-      <c r="E16" s="76" t="s">
-        <v>124</v>
-      </c>
-      <c r="F16" s="71">
-        <v>1</v>
-      </c>
-      <c r="G16" s="71" t="s">
-        <v>76</v>
-      </c>
-      <c r="H16" s="71" t="s">
-        <v>13</v>
-      </c>
-      <c r="I16" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="J16" s="71" t="s">
-        <v>47</v>
-      </c>
-      <c r="K16" s="78" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="210" x14ac:dyDescent="0.25">
-      <c r="A17" s="70" t="s">
-        <v>68</v>
-      </c>
-      <c r="B17" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="C17" s="76" t="s">
-        <v>101</v>
-      </c>
-      <c r="D17" s="72" t="s">
-        <v>107</v>
-      </c>
-      <c r="E17" s="76" t="s">
-        <v>124</v>
-      </c>
-      <c r="F17" s="71">
-        <v>1</v>
-      </c>
-      <c r="G17" s="71" t="s">
-        <v>76</v>
-      </c>
-      <c r="H17" s="71" t="s">
-        <v>13</v>
-      </c>
-      <c r="I17" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="J17" s="71" t="s">
-        <v>47</v>
-      </c>
-      <c r="K17" s="78" t="s">
+      <c r="K20" s="57" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="210" x14ac:dyDescent="0.25">
-      <c r="A18" s="70" t="s">
-        <v>68</v>
-      </c>
-      <c r="B18" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" s="76" t="s">
-        <v>103</v>
-      </c>
-      <c r="D18" s="72" t="s">
-        <v>107</v>
-      </c>
-      <c r="E18" s="76" t="s">
-        <v>124</v>
-      </c>
-      <c r="F18" s="71">
-        <v>1</v>
-      </c>
-      <c r="G18" s="71" t="s">
-        <v>76</v>
-      </c>
-      <c r="H18" s="71" t="s">
-        <v>13</v>
-      </c>
-      <c r="I18" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="J18" s="71" t="s">
-        <v>47</v>
-      </c>
-      <c r="K18" s="78" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="70"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="70"/>
-    </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="70"/>
+      <c r="A21" s="49"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="70"/>
+      <c r="A22" s="49"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="70"/>
+      <c r="A23" s="49"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="70"/>
+      <c r="A24" s="49"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="70"/>
+      <c r="A25" s="49"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="70"/>
+      <c r="A26" s="49"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="70"/>
+      <c r="A27" s="49"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="70"/>
+      <c r="A28" s="49"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="70"/>
+      <c r="A29" s="49"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="70"/>
+      <c r="A30" s="49"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="70"/>
+      <c r="A31" s="49"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="70"/>
+      <c r="A32" s="49"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6865,430 +6745,600 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="21.28515625" style="73" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="73" customWidth="1"/>
-    <col min="4" max="4" width="58.5703125" style="77" customWidth="1"/>
-    <col min="5" max="5" width="33.85546875" style="74" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="2" width="21.28515625" style="52" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="52" customWidth="1"/>
+    <col min="4" max="4" width="58.5703125" style="56" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" style="53" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" style="52" customWidth="1"/>
+    <col min="7" max="7" width="58.5703125" style="56" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="63" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="61" t="s">
+    <row r="1" spans="1:7" s="42" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="61" t="s">
+      <c r="C1" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="62" t="s">
+      <c r="D1" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="E1" s="62" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="71" t="s">
+      <c r="E1" s="41" t="s">
+        <v>149</v>
+      </c>
+      <c r="F1" s="78" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="41" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="71" t="s">
+      <c r="B2" s="50" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="55" t="s">
+        <v>72</v>
+      </c>
+      <c r="E2" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F2" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="55"/>
+    </row>
+    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>125</v>
+      </c>
+      <c r="C3" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="55" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F3" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="55"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="50" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="55" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F4" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="55"/>
+    </row>
+    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="50" t="s">
+        <v>125</v>
+      </c>
+      <c r="C5" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="55" t="s">
+        <v>84</v>
+      </c>
+      <c r="E5" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F5" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="55"/>
+    </row>
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="50" t="s">
+        <v>125</v>
+      </c>
+      <c r="C6" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="55" t="s">
+        <v>86</v>
+      </c>
+      <c r="E6" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F6" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="55"/>
+    </row>
+    <row r="7" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="50" t="s">
+        <v>129</v>
+      </c>
+      <c r="C7" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="55" t="s">
+        <v>158</v>
+      </c>
+      <c r="E7" s="51" t="s">
+        <v>183</v>
+      </c>
+      <c r="F7" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="55"/>
+    </row>
+    <row r="8" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="50" t="s">
+        <v>129</v>
+      </c>
+      <c r="C8" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="55" t="s">
+        <v>159</v>
+      </c>
+      <c r="E8" s="51" t="s">
+        <v>183</v>
+      </c>
+      <c r="F8" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="55"/>
+    </row>
+    <row r="9" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="50" t="s">
+        <v>129</v>
+      </c>
+      <c r="C9" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="55" t="s">
+        <v>160</v>
+      </c>
+      <c r="E9" s="51" t="s">
+        <v>183</v>
+      </c>
+      <c r="F9" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="55"/>
+    </row>
+    <row r="10" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" s="50" t="s">
+        <v>129</v>
+      </c>
+      <c r="C10" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="55" t="s">
+        <v>161</v>
+      </c>
+      <c r="E10" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="F10" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="55"/>
+    </row>
+    <row r="11" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="C11" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="55" t="s">
+        <v>162</v>
+      </c>
+      <c r="E11" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F11" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="55"/>
+    </row>
+    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="C12" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="E12" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F12" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" s="55"/>
+    </row>
+    <row r="13" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="C13" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="55" t="s">
+        <v>164</v>
+      </c>
+      <c r="E13" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F13" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" s="55"/>
+    </row>
+    <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="C14" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="55" t="s">
+        <v>165</v>
+      </c>
+      <c r="E14" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F14" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="55"/>
+    </row>
+    <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="C15" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="55" t="s">
+        <v>166</v>
+      </c>
+      <c r="E15" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F15" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" s="55"/>
+    </row>
+    <row r="16" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="C16" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="55" t="s">
+        <v>167</v>
+      </c>
+      <c r="E16" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F16" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" s="55"/>
+    </row>
+    <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="C17" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="55" t="s">
+        <v>168</v>
+      </c>
+      <c r="E17" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="F17" s="52" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="55"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="50" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="71" t="s">
+      <c r="C18" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="76" t="s">
-        <v>72</v>
-      </c>
-      <c r="E2" s="72" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="71" t="s">
+      <c r="D18" s="55" t="s">
+        <v>169</v>
+      </c>
+      <c r="E18" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F18" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" s="55"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="71" t="s">
+      <c r="B19" s="50" t="s">
         <v>127</v>
       </c>
-      <c r="C3" s="71" t="s">
+      <c r="C19" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="76" t="s">
-        <v>73</v>
-      </c>
-      <c r="E3" s="72" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="71" t="s">
+      <c r="D19" s="55" t="s">
+        <v>170</v>
+      </c>
+      <c r="E19" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F19" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G19" s="55"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="71" t="s">
+      <c r="B20" s="50" t="s">
         <v>127</v>
       </c>
-      <c r="C4" s="71" t="s">
+      <c r="C20" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="76" t="s">
-        <v>79</v>
-      </c>
-      <c r="E4" s="72" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="71" t="s">
+      <c r="D20" s="55" t="s">
+        <v>171</v>
+      </c>
+      <c r="E20" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="F20" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" s="55"/>
+    </row>
+    <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="71" t="s">
-        <v>127</v>
-      </c>
-      <c r="C5" s="71" t="s">
+      <c r="B21" s="50" t="s">
+        <v>131</v>
+      </c>
+      <c r="C21" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="76" t="s">
-        <v>84</v>
-      </c>
-      <c r="E5" s="72" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="71" t="s">
+      <c r="D21" s="55" t="s">
+        <v>172</v>
+      </c>
+      <c r="E21" s="51" t="s">
+        <v>189</v>
+      </c>
+      <c r="F21" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G21" s="55" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="71" t="s">
-        <v>127</v>
-      </c>
-      <c r="C6" s="71" t="s">
+      <c r="B22" s="50" t="s">
+        <v>131</v>
+      </c>
+      <c r="C22" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="76" t="s">
-        <v>86</v>
-      </c>
-      <c r="E6" s="72" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" s="71" t="s">
+      <c r="D22" s="55" t="s">
+        <v>173</v>
+      </c>
+      <c r="E22" s="51" t="s">
+        <v>189</v>
+      </c>
+      <c r="F22" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="55" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="71" t="s">
+      <c r="B23" s="50" t="s">
         <v>131</v>
       </c>
-      <c r="C7" s="71" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="76" t="s">
-        <v>160</v>
-      </c>
-      <c r="E7" s="72" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A8" s="71" t="s">
+      <c r="C23" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="55" t="s">
+        <v>174</v>
+      </c>
+      <c r="E23" s="51" t="s">
+        <v>189</v>
+      </c>
+      <c r="F23" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="55" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="71" t="s">
+      <c r="B24" s="50" t="s">
         <v>131</v>
       </c>
-      <c r="C8" s="71" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="76" t="s">
-        <v>161</v>
-      </c>
-      <c r="E8" s="72" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" s="71" t="s">
+      <c r="C24" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="55" t="s">
+        <v>175</v>
+      </c>
+      <c r="E24" s="51" t="s">
+        <v>189</v>
+      </c>
+      <c r="F24" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="55" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="71" t="s">
+      <c r="B25" s="50" t="s">
         <v>131</v>
       </c>
-      <c r="C9" s="71" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="76" t="s">
-        <v>162</v>
-      </c>
-      <c r="E9" s="72" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A10" s="71" t="s">
+      <c r="C25" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="55" t="s">
+        <v>188</v>
+      </c>
+      <c r="E25" s="51" t="s">
+        <v>189</v>
+      </c>
+      <c r="F25" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="55" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="71" t="s">
+      <c r="B26" s="50" t="s">
         <v>131</v>
       </c>
-      <c r="C10" s="71" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="76" t="s">
-        <v>163</v>
-      </c>
-      <c r="E10" s="72" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11" s="71" t="s">
-        <v>132</v>
-      </c>
-      <c r="C11" s="71" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="76" t="s">
-        <v>164</v>
-      </c>
-      <c r="E11" s="72" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="71" t="s">
-        <v>132</v>
-      </c>
-      <c r="C12" s="71" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="76" t="s">
-        <v>165</v>
-      </c>
-      <c r="E12" s="72" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" s="71" t="s">
-        <v>132</v>
-      </c>
-      <c r="C13" s="71" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="76" t="s">
-        <v>166</v>
-      </c>
-      <c r="E13" s="72" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A14" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" s="71" t="s">
-        <v>132</v>
-      </c>
-      <c r="C14" s="71" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="76" t="s">
-        <v>167</v>
-      </c>
-      <c r="E14" s="72" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A15" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B15" s="71" t="s">
-        <v>132</v>
-      </c>
-      <c r="C15" s="71" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="76" t="s">
-        <v>168</v>
-      </c>
-      <c r="E15" s="72" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A16" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" s="71" t="s">
-        <v>132</v>
-      </c>
-      <c r="C16" s="71" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="76" t="s">
-        <v>169</v>
-      </c>
-      <c r="E16" s="72" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="71" t="s">
-        <v>132</v>
-      </c>
-      <c r="C17" s="71" t="s">
+      <c r="C26" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="76" t="s">
-        <v>170</v>
-      </c>
-      <c r="E17" s="72" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A18" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B18" s="71" t="s">
-        <v>129</v>
-      </c>
-      <c r="C18" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="D18" s="76" t="s">
-        <v>171</v>
-      </c>
-      <c r="E18" s="72" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A19" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B19" s="71" t="s">
-        <v>129</v>
-      </c>
-      <c r="C19" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" s="76" t="s">
-        <v>172</v>
-      </c>
-      <c r="E19" s="72" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A20" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="71" t="s">
-        <v>129</v>
-      </c>
-      <c r="C20" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="D20" s="76" t="s">
-        <v>173</v>
-      </c>
-      <c r="E20" s="72" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" s="71" t="s">
-        <v>133</v>
-      </c>
-      <c r="C21" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" s="76" t="s">
-        <v>174</v>
-      </c>
-      <c r="E21" s="72" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B22" s="71" t="s">
-        <v>133</v>
-      </c>
-      <c r="C22" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="D22" s="76" t="s">
-        <v>175</v>
-      </c>
-      <c r="E22" s="72" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A23" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" s="71" t="s">
-        <v>133</v>
-      </c>
-      <c r="C23" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="D23" s="76" t="s">
-        <v>176</v>
-      </c>
-      <c r="E23" s="72" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="B24" s="71" t="s">
-        <v>133</v>
-      </c>
-      <c r="C24" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="D24" s="76" t="s">
-        <v>177</v>
-      </c>
-      <c r="E24" s="72" t="s">
-        <v>107</v>
+      <c r="D26" s="55" t="s">
+        <v>187</v>
+      </c>
+      <c r="E26" s="51" t="s">
+        <v>189</v>
+      </c>
+      <c r="F26" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="55" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E1:E1048576">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"Failed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"Passed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+      <formula>"N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E1048576" xr:uid="{0A0ED6EF-873A-4559-A681-3F531C79522E}">
+      <formula1>"Passed,Failed,In Progress,Not Started,N/A,"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DCE03FCA-DB1E-470A-A8AC-6ACD3F53F6BB}">
           <x14:formula1>
             <xm:f>'Brainstorm Flow'!$A$2:$A$35</xm:f>
@@ -7306,6 +7356,12 @@
             <xm:f>'Brainstorm Flow'!$B$2:$B$8</xm:f>
           </x14:formula1>
           <xm:sqref>B2:C1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A3A96FB6-E4EE-4380-9E12-8ABE5EDB7238}">
+          <x14:formula1>
+            <xm:f>Legends!$B$2:$B$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>F1:F16 F18:F1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -7329,19 +7385,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="65" t="s">
+      <c r="B1" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="65" t="s">
+      <c r="C1" s="44" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="65" t="s">
+      <c r="D1" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="65" t="s">
+      <c r="E1" s="44" t="s">
         <v>34</v>
       </c>
     </row>
@@ -7358,7 +7414,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>16</v>
@@ -7366,7 +7422,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>16</v>
@@ -7403,55 +7459,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="43" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="43" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="64" t="s">
-        <v>130</v>
-      </c>
-      <c r="C1" s="64" t="s">
+      <c r="C1" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="D1" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="E1" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="64" t="s">
-        <v>140</v>
-      </c>
-      <c r="E1" s="64" t="s">
+      <c r="F1" s="43" t="s">
         <v>141</v>
-      </c>
-      <c r="F1" s="64" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>70</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>20</v>
@@ -7463,34 +7519,34 @@
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
-      <c r="B7" s="80" t="s">
-        <v>134</v>
+      <c r="B7" s="59" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="80" t="s">
-        <v>135</v>
+      <c r="B8" s="59" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>